<commit_message>
live update 19:17:57 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-tnt-ursa-2026-04-02_20260402_191249.xlsx
+++ b/data/live_logs/live_cs2-tnt-ursa-2026-04-02_20260402_191249.xlsx
@@ -66,7 +66,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -75,6 +75,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -440,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD2"/>
+  <dimension ref="A1:AD4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -454,7 +455,7 @@
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="9" customWidth="1" min="10" max="10"/>
     <col width="9" customWidth="1" min="11" max="11"/>
-    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
     <col width="9" customWidth="1" min="15" max="15"/>
@@ -470,7 +471,7 @@
     <col width="23" customWidth="1" min="25" max="25"/>
     <col width="14" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
-    <col width="27" customWidth="1" min="28" max="28"/>
+    <col width="30" customWidth="1" min="28" max="28"/>
     <col width="8" customWidth="1" min="29" max="29"/>
     <col width="8" customWidth="1" min="30" max="30"/>
   </cols>
@@ -736,6 +737,231 @@
         </is>
       </c>
       <c r="AD2" t="inlineStr">
+        <is>
+          <t>TNT</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>19:14:26</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>dust2</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>16</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>12-4</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>0.9752999999999999</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>0.4876</v>
+      </c>
+      <c r="J3" t="n">
+        <v>4000</v>
+      </c>
+      <c r="K3" t="n">
+        <v>7300</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>50</v>
+      </c>
+      <c r="O3" t="n">
+        <v>40</v>
+      </c>
+      <c r="P3" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>6</v>
+      </c>
+      <c r="R3" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S3" s="2" t="n">
+        <v>0.655</v>
+      </c>
+      <c r="T3" s="2" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="U3" s="2" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="V3" t="n">
+        <v>22517.2315</v>
+      </c>
+      <c r="X3" s="2" t="n">
+        <v>-0.01473366260528561</v>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z3" t="n">
+        <v>29.92</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>33.51</v>
+      </c>
+      <c r="AB3" s="4" t="inlineStr">
+        <is>
+          <t>SELL WINNER Ursa P/L:$+29.92</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>TNT</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>19:15:51</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>dust2</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>17</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>13-4</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>0.9911</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>0.9911</v>
+      </c>
+      <c r="J4" t="n">
+        <v>6750</v>
+      </c>
+      <c r="K4" t="n">
+        <v>7100</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>55</v>
+      </c>
+      <c r="O4" t="n">
+        <v>41</v>
+      </c>
+      <c r="P4" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>6</v>
+      </c>
+      <c r="R4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S4" s="2" t="n">
+        <v>0.655</v>
+      </c>
+      <c r="T4" s="2" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="U4" s="2" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="V4" t="n">
+        <v>22517.2315</v>
+      </c>
+      <c r="W4" s="3" t="n">
+        <v>0.601124153137207</v>
+      </c>
+      <c r="X4" s="2" t="n">
+        <v>0.001124153137207068</v>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>WINNER:Ursa@0.360x278</t>
+        </is>
+      </c>
+      <c r="Z4" t="n">
+        <v>29.92</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB4" s="4" t="inlineStr">
+        <is>
+          <t>BUY WINNER Ursa $100@0.360</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
         <is>
           <t>TNT</t>
         </is>
@@ -752,7 +978,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -766,8 +992,8 @@
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="21" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="21" customWidth="1" min="12" max="12"/>
-    <col width="5" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -885,6 +1111,108 @@
         <v>0.10513378739357</v>
       </c>
       <c r="M2" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>19:14:26</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>16</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>dust2</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>WINNER</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>119.6944444444445</v>
+      </c>
+      <c r="I3" s="6" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="J3" s="6" t="n">
+        <v>0.4876331686973572</v>
+      </c>
+      <c r="K3" s="6" t="n">
+        <v>0.655</v>
+      </c>
+      <c r="L3" s="6" t="n">
+        <v>-0.1523668313026428</v>
+      </c>
+      <c r="M3" s="8" t="n">
+        <v>29.92361111111111</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>19:15:51</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>17</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>dust2</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>WINNER</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>277.7777777777778</v>
+      </c>
+      <c r="I4" s="6" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="J4" s="6" t="n">
+        <v>0.991124153137207</v>
+      </c>
+      <c r="K4" s="6" t="n">
+        <v>0.655</v>
+      </c>
+      <c r="L4" s="6" t="n">
+        <v>0.601124153137207</v>
+      </c>
+      <c r="M4" s="7" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>